<commit_message>
PCA for wealth index
</commit_message>
<xml_diff>
--- a/outputs/pca_contributions.xlsx
+++ b/outputs/pca_contributions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Academic\Nutritional epidemiology projects\ferritin-anemia_diagnosis\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A66B54-9F36-4DE9-9472-D665A53F5DB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C712DF1-F5DB-4063-B99D-A5306CAD5258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,42 +20,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Dim.1</t>
   </si>
   <si>
-    <t>wall_brick</t>
-  </si>
-  <si>
-    <t>wall_adobe</t>
-  </si>
-  <si>
-    <t>roof_concrete</t>
-  </si>
-  <si>
-    <t>water_network</t>
-  </si>
-  <si>
-    <t>toilet_flush</t>
+    <t>roof_noble</t>
+  </si>
+  <si>
+    <t>roof_basic</t>
+  </si>
+  <si>
+    <t>wall_noble</t>
+  </si>
+  <si>
+    <t>toilet_safe</t>
   </si>
   <si>
     <t>floor_noble</t>
   </si>
   <si>
-    <t>room_none</t>
-  </si>
-  <si>
-    <t>water_truck</t>
-  </si>
-  <si>
-    <t>room_three_plus</t>
+    <t>room_two_plus</t>
+  </si>
+  <si>
+    <t>room_min</t>
+  </si>
+  <si>
+    <t>floor_basic</t>
+  </si>
+  <si>
+    <t>water_safe</t>
   </si>
   <si>
     <t>fuel_clean</t>
-  </si>
-  <si>
-    <t>toilet_none</t>
   </si>
   <si>
     <t>light_electric</t>
@@ -430,11 +427,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="21.5703125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
@@ -446,7 +440,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>21.951804318321543</v>
+        <v>19.197790658699095</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -454,7 +448,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>20.421821655415346</v>
+        <v>19.028949442585898</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -462,7 +456,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>19.025090710339136</v>
+        <v>12.812621013926373</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -470,7 +464,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>10.677225322960222</v>
+        <v>10.053992211625333</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -478,7 +472,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>7.5489422539319877</v>
+        <v>9.8360356704010794</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -486,7 +480,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>6.7950947619490991</v>
+        <v>9.0117457990091427</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -494,7 +488,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>3.9564104629404677</v>
+        <v>9.0117457990091339</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -502,7 +496,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>3.9142226852036148</v>
+        <v>5.2273565491314997</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -510,7 +504,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>2.8180284601157219</v>
+        <v>5.1860594268731397</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -518,7 +512,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1.8425956593598061</v>
+        <v>0.48599500796908024</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -526,15 +520,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0.54600800210359723</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>0.5027557073594533</v>
+        <v>0.14770842077023316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>